<commit_message>
Updated mistaken coordinates Amsterdam
 Galileiplantsoen (#11)
</commit_message>
<xml_diff>
--- a/InstrumentList_v1.1.xlsx
+++ b/InstrumentList_v1.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\ESG\DOW_MAQ\MAQ_Archive\MAQ-Observations.nl\Admin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C003F57-41C8-416E-8784-AE0B42A67934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A195B0FB-19E8-48E6-9E57-455C1D3300BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-6645" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{F886D0CD-42D9-4E67-83C9-C1370524BEBE}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{F886D0CD-42D9-4E67-83C9-C1370524BEBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Veenkampen" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4896" uniqueCount="1059">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4898" uniqueCount="1060">
   <si>
     <t>Stream name</t>
   </si>
@@ -3468,9 +3468,6 @@
     <t>Tweede Oosterparkstraat (52.35675,4.91571)</t>
   </si>
   <si>
-    <t>Galileiplantsoen (52.31726,4.94016)</t>
-  </si>
-  <si>
     <t>DN_TA_10_1_1</t>
   </si>
   <si>
@@ -3910,6 +3907,12 @@
   </si>
   <si>
     <t>Updated MeasurementInterval for several streams</t>
+  </si>
+  <si>
+    <t>Galileiplantsoen (52.35382, 4.94016)</t>
+  </si>
+  <si>
+    <t>Corrected wrong coordinates for Galileiplantsoen (#11)</t>
   </si>
 </sst>
 </file>
@@ -8658,7 +8661,7 @@
         <v>728</v>
       </c>
       <c r="G213" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.25">
@@ -8681,27 +8684,27 @@
         <v>728</v>
       </c>
       <c r="G214" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B215" s="4" t="s">
         <v>351</v>
       </c>
       <c r="C215" s="4" t="s">
+        <v>1005</v>
+      </c>
+      <c r="D215" s="4" t="s">
         <v>1006</v>
       </c>
-      <c r="D215" s="4" t="s">
-        <v>1007</v>
-      </c>
       <c r="F215" t="s">
         <v>724</v>
       </c>
       <c r="G215" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
   </sheetData>
@@ -14534,7 +14537,7 @@
     </row>
     <row r="298" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="B298" s="4" t="s">
         <v>351</v>
@@ -14543,10 +14546,10 @@
         <v>725</v>
       </c>
       <c r="D298" s="4" t="s">
+        <v>1046</v>
+      </c>
+      <c r="E298" s="4" t="s">
         <v>1047</v>
-      </c>
-      <c r="E298" s="4" t="s">
-        <v>1048</v>
       </c>
       <c r="F298" t="s">
         <v>724</v>
@@ -14557,19 +14560,19 @@
     </row>
     <row r="299" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="B299" s="4" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="C299" s="4" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="D299" s="4" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="E299" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="F299" t="s">
         <v>724</v>
@@ -14580,19 +14583,19 @@
     </row>
     <row r="300" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="B300" s="4" t="s">
         <v>353</v>
       </c>
       <c r="C300" s="4" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="D300" s="4" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="E300" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="F300" t="s">
         <v>724</v>
@@ -14603,19 +14606,19 @@
     </row>
     <row r="301" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="B301" s="4" t="s">
         <v>353</v>
       </c>
       <c r="C301" s="4" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="D301" s="4" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="E301" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="F301" t="s">
         <v>724</v>
@@ -14626,19 +14629,19 @@
     </row>
     <row r="302" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B302" s="4" t="s">
         <v>353</v>
       </c>
       <c r="C302" s="4" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="D302" s="4" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="E302" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="F302" t="s">
         <v>724</v>
@@ -14649,19 +14652,19 @@
     </row>
     <row r="303" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="B303" s="4" t="s">
         <v>353</v>
       </c>
       <c r="C303" s="4" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="D303" s="4" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="E303" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="F303" t="s">
         <v>724</v>
@@ -14672,19 +14675,19 @@
     </row>
     <row r="304" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B304" s="4" t="s">
         <v>353</v>
       </c>
       <c r="C304" s="4" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="D304" s="4" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="E304" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="F304" t="s">
         <v>724</v>
@@ -14695,19 +14698,19 @@
     </row>
     <row r="305" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B305" s="4" t="s">
         <v>353</v>
       </c>
       <c r="C305" s="4" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="D305" s="4" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="E305" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="F305" t="s">
         <v>724</v>
@@ -14718,19 +14721,19 @@
     </row>
     <row r="306" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="B306" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C306" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="D306" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="E306" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="F306" t="s">
         <v>724</v>
@@ -14741,19 +14744,19 @@
     </row>
     <row r="307" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B307" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C307" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="D307" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="E307" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="F307" t="s">
         <v>724</v>
@@ -14764,19 +14767,19 @@
     </row>
     <row r="308" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="B308" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C308" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="D308" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="E308" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="F308" t="s">
         <v>724</v>
@@ -14787,19 +14790,19 @@
     </row>
     <row r="309" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B309" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C309" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="D309" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="E309" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="F309" t="s">
         <v>724</v>
@@ -14810,19 +14813,19 @@
     </row>
     <row r="310" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="B310" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C310" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="D310" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="E310" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="F310" t="s">
         <v>724</v>
@@ -14833,19 +14836,19 @@
     </row>
     <row r="311" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B311" s="4" t="s">
         <v>362</v>
       </c>
       <c r="C311" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="D311" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="E311" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="F311" t="s">
         <v>724</v>
@@ -17666,10 +17669,10 @@
         <v>876</v>
       </c>
       <c r="F142" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G142" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.25">
@@ -17689,10 +17692,10 @@
         <v>876</v>
       </c>
       <c r="F143" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G143" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.25">
@@ -17712,10 +17715,10 @@
         <v>875</v>
       </c>
       <c r="F144" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G144" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.25">
@@ -17735,10 +17738,10 @@
         <v>875</v>
       </c>
       <c r="F145" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G145" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="146" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -17758,10 +17761,10 @@
         <v>875</v>
       </c>
       <c r="F146" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G146" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.25">
@@ -17784,7 +17787,7 @@
         <v>724</v>
       </c>
       <c r="G147" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="148" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -17807,7 +17810,7 @@
         <v>724</v>
       </c>
       <c r="G148" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.25">
@@ -17827,10 +17830,10 @@
         <v>908</v>
       </c>
       <c r="F149" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G149" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.25">
@@ -17850,10 +17853,10 @@
         <v>908</v>
       </c>
       <c r="F150" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G150" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.25">
@@ -17873,10 +17876,10 @@
         <v>908</v>
       </c>
       <c r="F151" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G151" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="152" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -17896,10 +17899,10 @@
         <v>908</v>
       </c>
       <c r="F152" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G152" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.25">
@@ -17922,7 +17925,7 @@
         <v>724</v>
       </c>
       <c r="G153" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="154" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -17945,7 +17948,7 @@
         <v>724</v>
       </c>
       <c r="G154" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.25">
@@ -17965,10 +17968,10 @@
         <v>874</v>
       </c>
       <c r="F155" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G155" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.25">
@@ -17988,10 +17991,10 @@
         <v>874</v>
       </c>
       <c r="F156" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G156" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.25">
@@ -18011,10 +18014,10 @@
         <v>874</v>
       </c>
       <c r="F157" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G157" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="158" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18034,10 +18037,10 @@
         <v>874</v>
       </c>
       <c r="F158" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G158" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="159" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18060,7 +18063,7 @@
         <v>724</v>
       </c>
       <c r="G159" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="160" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18083,7 +18086,7 @@
         <v>724</v>
       </c>
       <c r="G160" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.25">
@@ -18103,10 +18106,10 @@
         <v>873</v>
       </c>
       <c r="F161" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G161" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.25">
@@ -18126,10 +18129,10 @@
         <v>873</v>
       </c>
       <c r="F162" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G162" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="163" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18149,10 +18152,10 @@
         <v>873</v>
       </c>
       <c r="F163" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G163" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="164" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18175,7 +18178,7 @@
         <v>724</v>
       </c>
       <c r="G164" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="165" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18198,7 +18201,7 @@
         <v>724</v>
       </c>
       <c r="G165" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.25">
@@ -18218,10 +18221,10 @@
         <v>909</v>
       </c>
       <c r="F166" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G166" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.25">
@@ -18241,10 +18244,10 @@
         <v>909</v>
       </c>
       <c r="F167" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G167" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.25">
@@ -18264,10 +18267,10 @@
         <v>909</v>
       </c>
       <c r="F168" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G168" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="169" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18287,10 +18290,10 @@
         <v>909</v>
       </c>
       <c r="F169" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G169" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="170" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18313,7 +18316,7 @@
         <v>724</v>
       </c>
       <c r="G170" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="171" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18336,7 +18339,7 @@
         <v>724</v>
       </c>
       <c r="G171" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.25">
@@ -18356,10 +18359,10 @@
         <v>883</v>
       </c>
       <c r="F172" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G172" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.25">
@@ -18379,10 +18382,10 @@
         <v>883</v>
       </c>
       <c r="F173" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G173" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="174" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18402,10 +18405,10 @@
         <v>883</v>
       </c>
       <c r="F174" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G174" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="175" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18428,7 +18431,7 @@
         <v>724</v>
       </c>
       <c r="G175" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="176" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18451,7 +18454,7 @@
         <v>724</v>
       </c>
       <c r="G176" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="177" spans="1:7" x14ac:dyDescent="0.25">
@@ -18471,10 +18474,10 @@
         <v>896</v>
       </c>
       <c r="F177" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G177" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.25">
@@ -18494,10 +18497,10 @@
         <v>896</v>
       </c>
       <c r="F178" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G178" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="179" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18517,10 +18520,10 @@
         <v>896</v>
       </c>
       <c r="F179" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G179" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="180" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18543,7 +18546,7 @@
         <v>724</v>
       </c>
       <c r="G180" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="181" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18566,7 +18569,7 @@
         <v>724</v>
       </c>
       <c r="G181" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="182" spans="1:7" x14ac:dyDescent="0.25">
@@ -18589,7 +18592,7 @@
         <v>728</v>
       </c>
       <c r="G182" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="183" spans="1:7" x14ac:dyDescent="0.25">
@@ -18612,7 +18615,7 @@
         <v>728</v>
       </c>
       <c r="G183" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="184" spans="1:7" x14ac:dyDescent="0.25">
@@ -18632,10 +18635,10 @@
         <v>904</v>
       </c>
       <c r="F184" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G184" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.25">
@@ -18655,10 +18658,10 @@
         <v>904</v>
       </c>
       <c r="F185" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G185" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="186" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18678,10 +18681,10 @@
         <v>904</v>
       </c>
       <c r="F186" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G186" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="187" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18704,7 +18707,7 @@
         <v>724</v>
       </c>
       <c r="G187" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="188" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
@@ -18727,12 +18730,12 @@
         <v>724</v>
       </c>
       <c r="G188" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="B189" s="4" t="s">
         <v>347</v>
@@ -18747,15 +18750,15 @@
         <v>910</v>
       </c>
       <c r="F189" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G189" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="B190" s="4" t="s">
         <v>348</v>
@@ -18770,15 +18773,15 @@
         <v>910</v>
       </c>
       <c r="F190" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G190" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="191" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="B191" s="4" t="s">
         <v>361</v>
@@ -18793,15 +18796,15 @@
         <v>910</v>
       </c>
       <c r="F191" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G191" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="192" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="B192" s="4" t="s">
         <v>361</v>
@@ -18819,12 +18822,12 @@
         <v>724</v>
       </c>
       <c r="G192" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="193" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="B193" s="4" t="s">
         <v>361</v>
@@ -18842,12 +18845,12 @@
         <v>724</v>
       </c>
       <c r="G193" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="B194" s="4" t="s">
         <v>347</v>
@@ -18859,18 +18862,18 @@
         <v>877</v>
       </c>
       <c r="E194" t="s">
-        <v>911</v>
+        <v>1058</v>
       </c>
       <c r="F194" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G194" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="B195" s="4" t="s">
         <v>348</v>
@@ -18882,18 +18885,18 @@
         <v>878</v>
       </c>
       <c r="E195" t="s">
-        <v>911</v>
+        <v>1058</v>
       </c>
       <c r="F195" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G195" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="196" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="B196" s="4" t="s">
         <v>361</v>
@@ -18905,18 +18908,18 @@
         <v>879</v>
       </c>
       <c r="E196" t="s">
-        <v>911</v>
+        <v>1058</v>
       </c>
       <c r="F196" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G196" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="197" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="B197" s="4" t="s">
         <v>361</v>
@@ -18928,18 +18931,18 @@
         <v>880</v>
       </c>
       <c r="E197" t="s">
-        <v>911</v>
+        <v>1058</v>
       </c>
       <c r="F197" t="s">
         <v>724</v>
       </c>
       <c r="G197" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="198" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="B198" s="4" t="s">
         <v>361</v>
@@ -18951,18 +18954,18 @@
         <v>881</v>
       </c>
       <c r="E198" t="s">
-        <v>911</v>
+        <v>1058</v>
       </c>
       <c r="F198" t="s">
         <v>724</v>
       </c>
       <c r="G198" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="B199" s="4" t="s">
         <v>347</v>
@@ -18974,18 +18977,18 @@
         <v>877</v>
       </c>
       <c r="E199" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="F199" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G199" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="B200" s="4" t="s">
         <v>348</v>
@@ -18997,18 +19000,18 @@
         <v>878</v>
       </c>
       <c r="E200" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="F200" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G200" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="B201" s="4" t="s">
         <v>347</v>
@@ -19020,18 +19023,18 @@
         <v>882</v>
       </c>
       <c r="E201" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="F201" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G201" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="202" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="B202" s="4" t="s">
         <v>361</v>
@@ -19043,18 +19046,18 @@
         <v>879</v>
       </c>
       <c r="E202" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="F202" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G202" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="203" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="B203" s="4" t="s">
         <v>361</v>
@@ -19066,18 +19069,18 @@
         <v>880</v>
       </c>
       <c r="E203" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="F203" t="s">
         <v>724</v>
       </c>
       <c r="G203" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="204" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="B204" s="4" t="s">
         <v>361</v>
@@ -19089,18 +19092,18 @@
         <v>881</v>
       </c>
       <c r="E204" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="F204" t="s">
         <v>724</v>
       </c>
       <c r="G204" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B205" s="4" t="s">
         <v>347</v>
@@ -19112,18 +19115,18 @@
         <v>877</v>
       </c>
       <c r="E205" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="F205" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G205" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B206" s="4" t="s">
         <v>348</v>
@@ -19135,18 +19138,18 @@
         <v>878</v>
       </c>
       <c r="E206" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="F206" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G206" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="207" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="B207" s="4" t="s">
         <v>361</v>
@@ -19158,18 +19161,18 @@
         <v>879</v>
       </c>
       <c r="E207" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="F207" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G207" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="208" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B208" s="4" t="s">
         <v>361</v>
@@ -19181,18 +19184,18 @@
         <v>880</v>
       </c>
       <c r="E208" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="F208" t="s">
         <v>724</v>
       </c>
       <c r="G208" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="209" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B209" s="4" t="s">
         <v>361</v>
@@ -19204,18 +19207,18 @@
         <v>881</v>
       </c>
       <c r="E209" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="F209" t="s">
         <v>724</v>
       </c>
       <c r="G209" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B210" s="4" t="s">
         <v>347</v>
@@ -19227,18 +19230,18 @@
         <v>877</v>
       </c>
       <c r="E210" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="F210" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G210" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B211" s="4" t="s">
         <v>348</v>
@@ -19250,18 +19253,18 @@
         <v>878</v>
       </c>
       <c r="E211" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="F211" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G211" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="212" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B212" s="4" t="s">
         <v>361</v>
@@ -19273,18 +19276,18 @@
         <v>879</v>
       </c>
       <c r="E212" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="F212" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G212" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="213" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>955</v>
+        <v>954</v>
       </c>
       <c r="B213" s="4" t="s">
         <v>361</v>
@@ -19296,18 +19299,18 @@
         <v>880</v>
       </c>
       <c r="E213" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="F213" t="s">
         <v>724</v>
       </c>
       <c r="G213" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="214" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="B214" s="4" t="s">
         <v>361</v>
@@ -19319,18 +19322,18 @@
         <v>881</v>
       </c>
       <c r="E214" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="F214" t="s">
         <v>724</v>
       </c>
       <c r="G214" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="B215" s="4" t="s">
         <v>347</v>
@@ -19342,18 +19345,18 @@
         <v>877</v>
       </c>
       <c r="E215" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="F215" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G215" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="B216" s="4" t="s">
         <v>348</v>
@@ -19365,18 +19368,18 @@
         <v>878</v>
       </c>
       <c r="E216" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="F216" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G216" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="B217" s="4" t="s">
         <v>347</v>
@@ -19388,18 +19391,18 @@
         <v>882</v>
       </c>
       <c r="E217" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="F217" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G217" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="218" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="B218" s="4" t="s">
         <v>361</v>
@@ -19411,18 +19414,18 @@
         <v>879</v>
       </c>
       <c r="E218" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="F218" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G218" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="219" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
       <c r="B219" s="4" t="s">
         <v>361</v>
@@ -19434,18 +19437,18 @@
         <v>880</v>
       </c>
       <c r="E219" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="F219" t="s">
         <v>724</v>
       </c>
       <c r="G219" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="220" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="B220" s="4" t="s">
         <v>361</v>
@@ -19457,18 +19460,18 @@
         <v>881</v>
       </c>
       <c r="E220" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="F220" t="s">
         <v>724</v>
       </c>
       <c r="G220" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B221" s="4" t="s">
         <v>347</v>
@@ -19480,18 +19483,18 @@
         <v>877</v>
       </c>
       <c r="E221" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="F221" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G221" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B222" s="4" t="s">
         <v>348</v>
@@ -19503,18 +19506,18 @@
         <v>878</v>
       </c>
       <c r="E222" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="F222" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G222" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="223" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
       <c r="B223" s="4" t="s">
         <v>361</v>
@@ -19526,18 +19529,18 @@
         <v>879</v>
       </c>
       <c r="E223" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="F223" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G223" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="224" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B224" s="4" t="s">
         <v>361</v>
@@ -19549,18 +19552,18 @@
         <v>880</v>
       </c>
       <c r="E224" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="F224" t="s">
         <v>724</v>
       </c>
       <c r="G224" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="225" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B225" s="4" t="s">
         <v>361</v>
@@ -19572,18 +19575,18 @@
         <v>881</v>
       </c>
       <c r="E225" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="F225" t="s">
         <v>724</v>
       </c>
       <c r="G225" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B226" s="4" t="s">
         <v>347</v>
@@ -19595,18 +19598,18 @@
         <v>877</v>
       </c>
       <c r="E226" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="F226" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G226" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="B227" s="4" t="s">
         <v>348</v>
@@ -19618,18 +19621,18 @@
         <v>878</v>
       </c>
       <c r="E227" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="F227" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G227" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B228" s="4" t="s">
         <v>347</v>
@@ -19641,18 +19644,18 @@
         <v>882</v>
       </c>
       <c r="E228" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="F228" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G228" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="229" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B229" s="4" t="s">
         <v>361</v>
@@ -19664,18 +19667,18 @@
         <v>879</v>
       </c>
       <c r="E229" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="F229" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G229" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="230" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="B230" s="4" t="s">
         <v>361</v>
@@ -19687,18 +19690,18 @@
         <v>880</v>
       </c>
       <c r="E230" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="F230" t="s">
         <v>724</v>
       </c>
       <c r="G230" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="231" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="B231" s="4" t="s">
         <v>361</v>
@@ -19710,18 +19713,18 @@
         <v>881</v>
       </c>
       <c r="E231" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="F231" t="s">
         <v>724</v>
       </c>
       <c r="G231" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="B232" s="4" t="s">
         <v>347</v>
@@ -19733,18 +19736,18 @@
         <v>877</v>
       </c>
       <c r="E232" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="F232" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G232" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B233" s="4" t="s">
         <v>348</v>
@@ -19756,18 +19759,18 @@
         <v>878</v>
       </c>
       <c r="E233" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="F233" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G233" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="234" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B234" s="4" t="s">
         <v>361</v>
@@ -19779,18 +19782,18 @@
         <v>879</v>
       </c>
       <c r="E234" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="F234" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G234" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="235" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="B235" s="4" t="s">
         <v>361</v>
@@ -19802,18 +19805,18 @@
         <v>880</v>
       </c>
       <c r="E235" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="F235" t="s">
         <v>724</v>
       </c>
       <c r="G235" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="236" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B236" s="4" t="s">
         <v>361</v>
@@ -19825,18 +19828,18 @@
         <v>881</v>
       </c>
       <c r="E236" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="F236" t="s">
         <v>724</v>
       </c>
       <c r="G236" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="B237" s="4" t="s">
         <v>347</v>
@@ -19848,18 +19851,18 @@
         <v>877</v>
       </c>
       <c r="E237" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F237" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G237" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="B238" s="4" t="s">
         <v>348</v>
@@ -19871,18 +19874,18 @@
         <v>878</v>
       </c>
       <c r="E238" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F238" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G238" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="239" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B239" s="4" t="s">
         <v>361</v>
@@ -19894,18 +19897,18 @@
         <v>879</v>
       </c>
       <c r="E239" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F239" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G239" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="240" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="B240" s="4" t="s">
         <v>361</v>
@@ -19917,18 +19920,18 @@
         <v>880</v>
       </c>
       <c r="E240" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F240" t="s">
         <v>724</v>
       </c>
       <c r="G240" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="241" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B241" s="4" t="s">
         <v>361</v>
@@ -19940,18 +19943,18 @@
         <v>881</v>
       </c>
       <c r="E241" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="F241" t="s">
         <v>724</v>
       </c>
       <c r="G241" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="242" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="B242" s="4" t="s">
         <v>347</v>
@@ -19963,18 +19966,18 @@
         <v>877</v>
       </c>
       <c r="E242" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="F242" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G242" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="243" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="B243" s="4" t="s">
         <v>348</v>
@@ -19986,18 +19989,18 @@
         <v>878</v>
       </c>
       <c r="E243" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="F243" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G243" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="244" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="B244" s="4" t="s">
         <v>361</v>
@@ -20009,18 +20012,18 @@
         <v>879</v>
       </c>
       <c r="E244" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="F244" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G244" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="245" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B245" s="4" t="s">
         <v>361</v>
@@ -20032,18 +20035,18 @@
         <v>880</v>
       </c>
       <c r="E245" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
       <c r="F245" t="s">
         <v>724</v>
       </c>
       <c r="G245" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="246" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="B246" s="4" t="s">
         <v>361</v>
@@ -20055,18 +20058,18 @@
         <v>881</v>
       </c>
       <c r="E246" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
       <c r="F246" t="s">
         <v>724</v>
       </c>
       <c r="G246" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="247" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="B247" s="4" t="s">
         <v>347</v>
@@ -20078,18 +20081,18 @@
         <v>877</v>
       </c>
       <c r="E247" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="F247" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G247" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="248" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="B248" s="4" t="s">
         <v>348</v>
@@ -20101,18 +20104,18 @@
         <v>878</v>
       </c>
       <c r="E248" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="F248" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G248" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="249" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="B249" s="4" t="s">
         <v>361</v>
@@ -20124,18 +20127,18 @@
         <v>879</v>
       </c>
       <c r="E249" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="F249" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G249" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="250" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="B250" s="4" t="s">
         <v>361</v>
@@ -20147,18 +20150,18 @@
         <v>880</v>
       </c>
       <c r="E250" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
       <c r="F250" t="s">
         <v>724</v>
       </c>
       <c r="G250" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="251" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B251" s="4" t="s">
         <v>361</v>
@@ -20170,18 +20173,18 @@
         <v>881</v>
       </c>
       <c r="E251" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="F251" t="s">
         <v>724</v>
       </c>
       <c r="G251" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="252" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="B252" s="4" t="s">
         <v>347</v>
@@ -20193,18 +20196,18 @@
         <v>877</v>
       </c>
       <c r="E252" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="F252" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G252" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="253" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="B253" s="4" t="s">
         <v>348</v>
@@ -20216,18 +20219,18 @@
         <v>878</v>
       </c>
       <c r="E253" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="F253" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G253" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="254" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B254" s="4" t="s">
         <v>361</v>
@@ -20239,18 +20242,18 @@
         <v>879</v>
       </c>
       <c r="E254" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="F254" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G254" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="255" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="B255" s="4" t="s">
         <v>361</v>
@@ -20262,18 +20265,18 @@
         <v>880</v>
       </c>
       <c r="E255" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="F255" t="s">
         <v>724</v>
       </c>
       <c r="G255" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="256" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B256" s="4" t="s">
         <v>361</v>
@@ -20285,18 +20288,18 @@
         <v>881</v>
       </c>
       <c r="E256" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="F256" t="s">
         <v>724</v>
       </c>
       <c r="G256" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B257" s="4" t="s">
         <v>347</v>
@@ -20308,18 +20311,18 @@
         <v>877</v>
       </c>
       <c r="E257" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="F257" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G257" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B258" s="4" t="s">
         <v>348</v>
@@ -20331,18 +20334,18 @@
         <v>878</v>
       </c>
       <c r="E258" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="F258" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G258" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="259" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="B259" s="4" t="s">
         <v>361</v>
@@ -20354,18 +20357,18 @@
         <v>879</v>
       </c>
       <c r="E259" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="F259" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="G259" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="260" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B260" s="4" t="s">
         <v>361</v>
@@ -20377,18 +20380,18 @@
         <v>880</v>
       </c>
       <c r="E260" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="F260" t="s">
         <v>724</v>
       </c>
       <c r="G260" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="261" spans="1:7" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B261" s="4" t="s">
         <v>361</v>
@@ -20400,13 +20403,13 @@
         <v>881</v>
       </c>
       <c r="E261" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="F261" t="s">
         <v>724</v>
       </c>
       <c r="G261" s="4" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
   </sheetData>
@@ -20419,7 +20422,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D9C5BFE-6C5D-49EF-B6DC-8FDF9610AF86}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
@@ -20514,7 +20517,7 @@
         <v>814</v>
       </c>
       <c r="B14" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -20522,19 +20525,19 @@
         <v>816</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="11" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="11" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -20558,27 +20561,27 @@
         <v>819</v>
       </c>
       <c r="B20" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B21" t="s">
         <v>1014</v>
-      </c>
-      <c r="B21" t="s">
-        <v>1015</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -20594,13 +20597,13 @@
         <v>818</v>
       </c>
       <c r="B25" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
@@ -20834,7 +20837,7 @@
         <v>740</v>
       </c>
       <c r="D46" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -20845,7 +20848,7 @@
         <v>740</v>
       </c>
       <c r="D47" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
@@ -20856,7 +20859,7 @@
         <v>740</v>
       </c>
       <c r="D48" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
@@ -20867,7 +20870,7 @@
         <v>740</v>
       </c>
       <c r="D49" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
@@ -20878,7 +20881,18 @@
         <v>740</v>
       </c>
       <c r="D50" t="s">
-        <v>1058</v>
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B51" s="10">
+        <v>46234</v>
+      </c>
+      <c r="C51" t="s">
+        <v>740</v>
+      </c>
+      <c r="D51" t="s">
+        <v>1059</v>
       </c>
     </row>
   </sheetData>

</xml_diff>